<commit_message>
add harvest params in default.params list
</commit_message>
<xml_diff>
--- a/scripts/params_scenarios.xlsx
+++ b/scripts/params_scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ctfccat-my.sharepoint.com/personal/nuria_aquilue_ctfc_cat/Documents/QBCMOD/AP-SBW/AP-SBW/scripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="197" documentId="8_{63479DC7-3D1F-4A2C-8933-2B9C44180743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{916F8845-11B3-4BA0-A73B-DF8670AA33F4}"/>
+  <xr:revisionPtr revIDLastSave="250" documentId="8_{63479DC7-3D1F-4A2C-8933-2B9C44180743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{669E9F09-AE4B-47D9-96F2-75953298AF9B}"/>
   <bookViews>
-    <workbookView xWindow="30330" yWindow="2430" windowWidth="17280" windowHeight="10050" activeTab="1" xr2:uid="{B274F7CD-F84C-4A76-ADBB-162A1E692C94}"/>
+    <workbookView xWindow="31980" yWindow="420" windowWidth="17280" windowHeight="10050" activeTab="1" xr2:uid="{B274F7CD-F84C-4A76-ADBB-162A1E692C94}"/>
   </bookViews>
   <sheets>
     <sheet name="param_dictionary" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="81">
   <si>
     <t>scenario</t>
   </si>
@@ -189,9 +189,6 @@
     <t>save.land.df</t>
   </si>
   <si>
-    <t>time.save</t>
-  </si>
-  <si>
     <t>Frequency in years to save the 'landscape' data frame</t>
   </si>
   <si>
@@ -204,9 +201,6 @@
     <t>Maximum number of neighbours in each bubble around the epicenters</t>
   </si>
   <si>
-    <t>Mean of a uniform distribution meaning the mid point of the spreading radius in the outbreak phase (in number of cells)</t>
-  </si>
-  <si>
     <t>Proportion of cells that are reduced to spread to in the preoubreak phase</t>
   </si>
   <si>
@@ -216,9 +210,6 @@
     <t>these are a number between 0 and 1 to indicate the reduction in number of cells that sbw does not actually spread</t>
   </si>
   <si>
-    <t>Range of a uniform distribution meaning the amplitud x 2 of the spreading radius in the outbreak phase (in number of cells)</t>
-  </si>
-  <si>
     <t>Default wind direction (º from N)</t>
   </si>
   <si>
@@ -256,6 +247,39 @@
   </si>
   <si>
     <t>stop.end.phase</t>
+  </si>
+  <si>
+    <t>freq.save</t>
+  </si>
+  <si>
+    <t>Mean of a uniform distribution meaning the mid point of the spreading radius in the outbreak phase (in km)</t>
+  </si>
+  <si>
+    <t>Range of a uniform distribution meaning the amplitud x 2 of the spreading radius in the outbreak phase (in km)</t>
+  </si>
+  <si>
+    <t>harv.rate</t>
+  </si>
+  <si>
+    <t>ap.rate</t>
+  </si>
+  <si>
+    <t>Artificial planting rate ([0,1])</t>
+  </si>
+  <si>
+    <t>Harvest rate ([0,1])</t>
+  </si>
+  <si>
+    <t>Black spruce regeneration rate ([0,1])</t>
+  </si>
+  <si>
+    <t>Trembling aspen regeneration rate ([0,1])</t>
+  </si>
+  <si>
+    <t>epn.rege.rate</t>
+  </si>
+  <si>
+    <t>pet.rege.rate</t>
   </si>
 </sst>
 </file>
@@ -299,19 +323,10 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -333,9 +348,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment textRotation="45"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment textRotation="45"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -344,6 +356,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment textRotation="45"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -360,6 +375,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -659,11 +678,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80EC21E7-99D0-4324-ADFF-33897A3E3BB6}">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="101.5546875" customWidth="1"/>
+    <col min="2" max="2" width="95.5546875" customWidth="1"/>
     <col min="3" max="3" width="13.33203125" style="3" customWidth="1"/>
     <col min="4" max="4" width="51.33203125" customWidth="1"/>
   </cols>
@@ -720,7 +739,7 @@
         <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>45</v>
@@ -728,10 +747,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" t="s">
         <v>50</v>
-      </c>
-      <c r="B6" t="s">
-        <v>51</v>
       </c>
       <c r="C6" s="3">
         <v>5</v>
@@ -739,7 +758,7 @@
     </row>
     <row r="7" spans="1:4" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
         <v>22</v>
@@ -769,7 +788,7 @@
       <c r="C9" s="3">
         <v>0</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>31</v>
       </c>
     </row>
@@ -783,7 +802,7 @@
       <c r="C10" s="3">
         <v>0</v>
       </c>
-      <c r="D10" s="8"/>
+      <c r="D10" s="7"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -795,7 +814,7 @@
       <c r="C11" s="3">
         <v>0</v>
       </c>
-      <c r="D11" s="8"/>
+      <c r="D11" s="7"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -807,7 +826,7 @@
       <c r="C12" s="3">
         <v>0</v>
       </c>
-      <c r="D12" s="8"/>
+      <c r="D12" s="7"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -861,7 +880,7 @@
         <v>37</v>
       </c>
       <c r="B17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C17" s="3">
         <v>200</v>
@@ -872,7 +891,7 @@
         <v>38</v>
       </c>
       <c r="B18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C18" s="3">
         <v>2000</v>
@@ -883,7 +902,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C19" s="3">
         <v>10</v>
@@ -894,7 +913,7 @@
         <v>40</v>
       </c>
       <c r="B20" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="C20" s="3">
         <v>5</v>
@@ -905,13 +924,13 @@
         <v>41</v>
       </c>
       <c r="B21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" s="3">
+        <v>0</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>56</v>
-      </c>
-      <c r="C21" s="3">
-        <v>0</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -919,19 +938,19 @@
         <v>42</v>
       </c>
       <c r="B22" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C22" s="3">
         <v>0</v>
       </c>
-      <c r="D22" s="9"/>
+      <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>43</v>
       </c>
       <c r="B23" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C23" s="3">
         <v>270</v>
@@ -942,7 +961,7 @@
         <v>11</v>
       </c>
       <c r="B24" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>44</v>
@@ -953,7 +972,7 @@
         <v>12</v>
       </c>
       <c r="B25" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C25" s="3">
         <v>0</v>
@@ -964,7 +983,7 @@
         <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C26" s="3">
         <v>40</v>
@@ -975,7 +994,7 @@
         <v>14</v>
       </c>
       <c r="B27" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C27" s="3">
         <v>0</v>
@@ -986,7 +1005,7 @@
         <v>15</v>
       </c>
       <c r="B28" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>46</v>
@@ -994,13 +1013,57 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B29" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>45</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>73</v>
+      </c>
+      <c r="B30" t="s">
+        <v>76</v>
+      </c>
+      <c r="C30" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>74</v>
+      </c>
+      <c r="B31" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>80</v>
+      </c>
+      <c r="B33" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" s="3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1014,14 +1077,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F70CED36-0713-4202-A98C-641A70715DBF}">
-  <dimension ref="A1:AC20"/>
+  <dimension ref="A1:AG20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="29" width="6.5546875" customWidth="1"/>
+    <col min="2" max="33" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="4" customFormat="1" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:33" s="4" customFormat="1" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
@@ -1037,10 +1100,10 @@
         <v>49</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>6</v>
@@ -1105,13 +1168,25 @@
       <c r="AB1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="AC1" s="6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AC1" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="AD1" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="AE1" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="AF1" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="AG1" s="9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B2" s="3">
         <v>2020</v>
@@ -1197,13 +1272,25 @@
       <c r="AC2" s="3" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AD2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B3" s="3">
-        <f t="shared" ref="B3:AC12" si="0">+B$2</f>
+        <f t="shared" ref="B3:AD12" si="0">+B$2</f>
         <v>2020</v>
       </c>
       <c r="C3" s="3">
@@ -1211,15 +1298,13 @@
         <v>1</v>
       </c>
       <c r="D3" s="3">
-        <v>4</v>
-      </c>
-      <c r="E3" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>FALSE</v>
+        <v>6</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>44</v>
       </c>
       <c r="F3" s="3">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G3" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1312,25 +1397,40 @@
         <f t="shared" si="0"/>
         <v>FALSE</v>
       </c>
-    </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AD3" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE3" s="3">
+        <f t="shared" ref="AD3:AG20" si="1">+AE$2</f>
+        <v>0</v>
+      </c>
+      <c r="AF3" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG3" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B4" s="3">
         <f t="shared" si="0"/>
         <v>2020</v>
       </c>
       <c r="C4" s="3">
-        <f t="shared" ref="C4" si="1">+C$2</f>
+        <f t="shared" ref="C4" si="2">+C$2</f>
         <v>1</v>
       </c>
       <c r="D4" s="3">
-        <v>4</v>
-      </c>
-      <c r="E4" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>FALSE</v>
+        <v>10</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="F4" s="3">
         <f t="shared" si="0"/>
@@ -1427,10 +1527,26 @@
         <f t="shared" si="0"/>
         <v>FALSE</v>
       </c>
-    </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AD4" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE4" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF4" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG4" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B5" s="3">
         <f t="shared" si="0"/>
@@ -1544,10 +1660,26 @@
         <f t="shared" si="0"/>
         <v>FALSE</v>
       </c>
-    </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AD5" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE5" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG5" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="str">
-        <f t="shared" ref="A6:P20" si="2">+A$2</f>
+        <f t="shared" ref="A6:P20" si="3">+A$2</f>
         <v>default</v>
       </c>
       <c r="B6" s="3">
@@ -1662,10 +1794,26 @@
         <f t="shared" si="0"/>
         <v>FALSE</v>
       </c>
-    </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AD6" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE6" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF6" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG6" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B7" s="3">
@@ -1780,10 +1928,26 @@
         <f t="shared" si="0"/>
         <v>FALSE</v>
       </c>
-    </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AD7" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE7" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF7" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG7" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B8" s="3">
@@ -1898,10 +2062,26 @@
         <f t="shared" si="0"/>
         <v>FALSE</v>
       </c>
-    </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AD8" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE8" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF8" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG8" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B9" s="3">
@@ -2016,10 +2196,26 @@
         <f t="shared" si="0"/>
         <v>FALSE</v>
       </c>
-    </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AD9" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE9" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF9" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG9" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B10" s="3">
@@ -2134,10 +2330,26 @@
         <f t="shared" si="0"/>
         <v>FALSE</v>
       </c>
-    </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AD10" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE10" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF10" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG10" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B11" s="3">
@@ -2252,10 +2464,26 @@
         <f t="shared" si="0"/>
         <v>FALSE</v>
       </c>
-    </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="AD11" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE11" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF11" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG11" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B12" s="3">
@@ -2271,1048 +2499,1192 @@
         <v>80</v>
       </c>
       <c r="E12" s="3" t="str">
-        <f t="shared" ref="E12:T20" si="3">+E$2</f>
+        <f t="shared" ref="E12:T20" si="4">+E$2</f>
         <v>FALSE</v>
       </c>
       <c r="F12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="G12" s="3" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>FALSE</v>
       </c>
       <c r="H12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>9</v>
       </c>
       <c r="I12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="J12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="L12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="M12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="N12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="O12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.6</v>
       </c>
       <c r="P12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.3</v>
       </c>
       <c r="Q12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>200</v>
       </c>
       <c r="R12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2000</v>
       </c>
       <c r="S12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="T12" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="U12" s="3">
-        <f t="shared" ref="U12:AC20" si="4">+U$2</f>
+        <f t="shared" ref="U12:AC20" si="5">+U$2</f>
         <v>0</v>
       </c>
       <c r="V12" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="W12" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>270</v>
       </c>
       <c r="X12" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>TRUE</v>
       </c>
       <c r="Y12" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Z12" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>40</v>
       </c>
       <c r="AA12" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AB12" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="AC12" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.3">
+        <f t="shared" si="5"/>
+        <v>FALSE</v>
+      </c>
+      <c r="AD12" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE12" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF12" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG12" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2020</v>
       </c>
       <c r="C13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="D13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>80</v>
       </c>
       <c r="E13" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="F13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="G13" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="H13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
       <c r="I13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.6</v>
       </c>
       <c r="P13" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.3</v>
       </c>
       <c r="Q13" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>200</v>
       </c>
       <c r="R13" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2000</v>
       </c>
       <c r="S13" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="T13" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="U13" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="V13" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="W13" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>270</v>
       </c>
       <c r="X13" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>TRUE</v>
       </c>
       <c r="Y13" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Z13" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>40</v>
       </c>
       <c r="AA13" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AB13" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="AC13" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.3">
+        <f t="shared" si="5"/>
+        <v>FALSE</v>
+      </c>
+      <c r="AD13" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE13" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF13" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG13" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2020</v>
       </c>
       <c r="C14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="D14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>80</v>
       </c>
       <c r="E14" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="F14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="G14" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="H14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
       <c r="I14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.6</v>
       </c>
       <c r="P14" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.3</v>
       </c>
       <c r="Q14" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>200</v>
       </c>
       <c r="R14" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2000</v>
       </c>
       <c r="S14" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="T14" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="U14" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="V14" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="W14" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>270</v>
       </c>
       <c r="X14" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>TRUE</v>
       </c>
       <c r="Y14" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Z14" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>40</v>
       </c>
       <c r="AA14" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AB14" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="AC14" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.3">
+        <f t="shared" si="5"/>
+        <v>FALSE</v>
+      </c>
+      <c r="AD14" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE14" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF14" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG14" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2020</v>
       </c>
       <c r="C15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="D15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>80</v>
       </c>
       <c r="E15" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="F15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="G15" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="H15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
       <c r="I15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.6</v>
       </c>
       <c r="P15" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.3</v>
       </c>
       <c r="Q15" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>200</v>
       </c>
       <c r="R15" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2000</v>
       </c>
       <c r="S15" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="T15" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="U15" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="V15" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="W15" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>270</v>
       </c>
       <c r="X15" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>TRUE</v>
       </c>
       <c r="Y15" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Z15" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>40</v>
       </c>
       <c r="AA15" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AB15" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="AC15" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.3">
+        <f t="shared" si="5"/>
+        <v>FALSE</v>
+      </c>
+      <c r="AD15" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE15" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF15" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG15" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2020</v>
       </c>
       <c r="C16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="D16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>80</v>
       </c>
       <c r="E16" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="F16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="G16" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="H16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
       <c r="I16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.6</v>
       </c>
       <c r="P16" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.3</v>
       </c>
       <c r="Q16" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>200</v>
       </c>
       <c r="R16" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2000</v>
       </c>
       <c r="S16" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="T16" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="U16" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="V16" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="W16" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>270</v>
       </c>
       <c r="X16" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>TRUE</v>
       </c>
       <c r="Y16" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Z16" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>40</v>
       </c>
       <c r="AA16" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AB16" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="AC16" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.3">
+        <f t="shared" si="5"/>
+        <v>FALSE</v>
+      </c>
+      <c r="AD16" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE16" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF16" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG16" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2020</v>
       </c>
       <c r="C17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="D17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>80</v>
       </c>
       <c r="E17" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="F17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="G17" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="H17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
       <c r="I17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.6</v>
       </c>
       <c r="P17" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.3</v>
       </c>
       <c r="Q17" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>200</v>
       </c>
       <c r="R17" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2000</v>
       </c>
       <c r="S17" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="T17" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="U17" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="V17" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="W17" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>270</v>
       </c>
       <c r="X17" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>TRUE</v>
       </c>
       <c r="Y17" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Z17" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>40</v>
       </c>
       <c r="AA17" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AB17" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="AC17" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.3">
+        <f t="shared" si="5"/>
+        <v>FALSE</v>
+      </c>
+      <c r="AD17" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE17" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF17" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG17" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2020</v>
       </c>
       <c r="C18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="D18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>80</v>
       </c>
       <c r="E18" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="F18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="G18" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="H18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
       <c r="I18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.6</v>
       </c>
       <c r="P18" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.3</v>
       </c>
       <c r="Q18" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>200</v>
       </c>
       <c r="R18" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2000</v>
       </c>
       <c r="S18" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="T18" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="U18" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="V18" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="W18" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>270</v>
       </c>
       <c r="X18" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>TRUE</v>
       </c>
       <c r="Y18" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Z18" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>40</v>
       </c>
       <c r="AA18" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AB18" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="AC18" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.3">
+        <f t="shared" si="5"/>
+        <v>FALSE</v>
+      </c>
+      <c r="AD18" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE18" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF18" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG18" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2020</v>
       </c>
       <c r="C19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="D19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>80</v>
       </c>
       <c r="E19" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="F19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="G19" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="H19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
       <c r="I19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.6</v>
       </c>
       <c r="P19" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.3</v>
       </c>
       <c r="Q19" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>200</v>
       </c>
       <c r="R19" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2000</v>
       </c>
       <c r="S19" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="T19" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="U19" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="V19" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="W19" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>270</v>
       </c>
       <c r="X19" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>TRUE</v>
       </c>
       <c r="Y19" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Z19" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>40</v>
       </c>
       <c r="AA19" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AB19" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="AC19" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.3">
+        <f t="shared" si="5"/>
+        <v>FALSE</v>
+      </c>
+      <c r="AD19" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE19" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF19" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG19" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>default</v>
       </c>
       <c r="B20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2020</v>
       </c>
       <c r="C20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="D20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>80</v>
       </c>
       <c r="E20" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="F20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="G20" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>FALSE</v>
       </c>
       <c r="H20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
       <c r="I20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="O20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.6</v>
       </c>
       <c r="P20" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.3</v>
       </c>
       <c r="Q20" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>200</v>
       </c>
       <c r="R20" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2000</v>
       </c>
       <c r="S20" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="T20" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="U20" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="V20" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="W20" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>270</v>
       </c>
       <c r="X20" s="3" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>TRUE</v>
       </c>
       <c r="Y20" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Z20" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>40</v>
       </c>
       <c r="AA20" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AB20" s="3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.5</v>
       </c>
       <c r="AC20" s="3" t="str">
-        <f t="shared" si="4"/>
-        <v>FALSE</v>
+        <f t="shared" si="5"/>
+        <v>FALSE</v>
+      </c>
+      <c r="AD20" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE20" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF20" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AG20" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>